<commit_message>
Add Load Demo Data button + richer demo-voters.xlsx
- app.html: Load Demo Data button + download link for demo-voters.xlsx
- app.js: fetch+parse demo XLSX via SheetJS, shared showResults()
- demo-voters.xlsx: 6 voters with Name/Phone/Ward/Year/Constituency
</commit_message>
<xml_diff>
--- a/public/demo-voters.xlsx
+++ b/public/demo-voters.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,6 +412,9 @@
       <c r="D1" t="str">
         <v>Year</v>
       </c>
+      <c r="E1" t="str">
+        <v>Constituency</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -426,6 +429,9 @@
       <c r="D2" t="str">
         <v>2024</v>
       </c>
+      <c r="E2" t="str">
+        <v>North</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -440,6 +446,9 @@
       <c r="D3" t="str">
         <v>2024</v>
       </c>
+      <c r="E3" t="str">
+        <v>North</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -454,6 +463,9 @@
       <c r="D4" t="str">
         <v>2024</v>
       </c>
+      <c r="E4" t="str">
+        <v>South</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -468,6 +480,9 @@
       <c r="D5" t="str">
         <v>2024</v>
       </c>
+      <c r="E5" t="str">
+        <v>North</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -482,6 +497,9 @@
       <c r="D6" t="str">
         <v>2024</v>
       </c>
+      <c r="E6" t="str">
+        <v>East</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -496,10 +514,13 @@
       <c r="D7" t="str">
         <v>2024</v>
       </c>
+      <c r="E7" t="str">
+        <v>South</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>